<commit_message>
Update the Risk Register to include Residual Risk
</commit_message>
<xml_diff>
--- a/Risk_Register_Cat_Cafe.xlsx
+++ b/Risk_Register_Cat_Cafe.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\airpl\Desktop\GRC_Work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{304F043A-3A33-49ED-9376-7EC77A7AC51C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA399CF-829D-42CD-AA4C-EA0AEC30C7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Legend" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="104">
   <si>
     <t>Description</t>
   </si>
@@ -185,9 +185,6 @@
     <t xml:space="preserve">Significant financial loss ( Higher than $25-75K ) </t>
   </si>
   <si>
-    <t>Mitigations</t>
-  </si>
-  <si>
     <t>Employees would be without pay for the duration of the system outage.</t>
   </si>
   <si>
@@ -297,6 +294,57 @@
   </si>
   <si>
     <t>Risk Owner</t>
+  </si>
+  <si>
+    <t>Residual Risk</t>
+  </si>
+  <si>
+    <t>Inherent Risk Score</t>
+  </si>
+  <si>
+    <t>Key Controls</t>
+  </si>
+  <si>
+    <t>Robust password policy, MFA</t>
+  </si>
+  <si>
+    <t>VLANs, Separate guest and Business Networks, WPA3</t>
+  </si>
+  <si>
+    <t>Encryption, Access Controls</t>
+  </si>
+  <si>
+    <t>MFA, Training</t>
+  </si>
+  <si>
+    <t>MFA, User training</t>
+  </si>
+  <si>
+    <t>Physical security, Patch Management</t>
+  </si>
+  <si>
+    <t>Access Controls</t>
+  </si>
+  <si>
+    <t>User Training</t>
+  </si>
+  <si>
+    <t>Third Party Risk Assessments and Audits</t>
+  </si>
+  <si>
+    <t>Access Controls, Encryption,</t>
+  </si>
+  <si>
+    <t>Business continuity planning</t>
+  </si>
+  <si>
+    <t>Business continuity planinng</t>
+  </si>
+  <si>
+    <t>EDR, Patch Management, Back-Ups, Disaster Recovery, Secure Data storage</t>
+  </si>
+  <si>
+    <t>Mitigation Notes</t>
   </si>
 </sst>
 </file>
@@ -871,7 +919,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45BDE1F6-370B-5145-B14B-5219F1CE6608}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr defaultColWidth="10.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.1796875" style="1" customWidth="1"/>
@@ -882,7 +930,9 @@
     <col min="6" max="6" width="18" style="1" customWidth="1"/>
     <col min="7" max="7" width="32.26953125" style="1" customWidth="1"/>
     <col min="8" max="8" width="54.81640625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="10.81640625" style="1"/>
+    <col min="9" max="9" width="43.453125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="39.1796875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="10.81640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -973,7 +1023,7 @@
     </row>
     <row r="10" spans="1:8" ht="20" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A10" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B10" s="24" t="s">
         <v>4</v>
@@ -993,7 +1043,7 @@
     </row>
     <row r="11" spans="1:8" ht="20" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A11" s="25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B11" s="26" t="s">
         <v>3</v>
@@ -1054,12 +1104,12 @@
       <c r="D15"/>
       <c r="E15"/>
     </row>
-    <row r="17" spans="1:8" ht="21" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:10" ht="21" x14ac:dyDescent="0.5">
       <c r="A17" s="29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B17" s="29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C17" s="29" t="s">
         <v>21</v>
@@ -1071,16 +1121,22 @@
         <v>22</v>
       </c>
       <c r="F17" s="29" t="s">
-        <v>11</v>
+        <v>88</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>50</v>
+        <v>87</v>
       </c>
       <c r="H17" s="29" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+      <c r="I17" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="J17" s="29" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>23</v>
       </c>
@@ -1088,25 +1144,31 @@
         <v>33</v>
       </c>
       <c r="C18" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="1">
         <v>2</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="F18" s="32">
-        <v>2</v>
-      </c>
-      <c r="G18" s="33" t="s">
-        <v>84</v>
+        <v>64</v>
+      </c>
+      <c r="F18" s="31">
+        <v>4</v>
+      </c>
+      <c r="G18" s="1">
+        <v>2</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+      <c r="I18" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>24</v>
       </c>
@@ -1120,19 +1182,25 @@
         <v>1</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F19" s="32">
         <v>2</v>
       </c>
-      <c r="G19" s="33" t="s">
-        <v>53</v>
+      <c r="G19" s="1">
+        <v>1</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+        <v>90</v>
+      </c>
+      <c r="I19" s="33" t="s">
+        <v>52</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>25</v>
       </c>
@@ -1146,19 +1214,25 @@
         <v>3</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F20" s="30">
         <v>6</v>
       </c>
-      <c r="G20" s="33" t="s">
-        <v>83</v>
+      <c r="G20" s="1">
+        <v>3</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+        <v>92</v>
+      </c>
+      <c r="I20" s="33" t="s">
+        <v>82</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>26</v>
       </c>
@@ -1172,19 +1246,25 @@
         <v>3</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F21" s="30">
         <v>9</v>
       </c>
-      <c r="G21" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="H21" s="33" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="G21" s="1">
+        <v>3</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I21" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="J21" s="33" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>27</v>
       </c>
@@ -1198,19 +1278,25 @@
         <v>3</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F22" s="31">
         <v>3</v>
       </c>
-      <c r="G22" s="33" t="s">
-        <v>82</v>
+      <c r="G22" s="1">
+        <v>3</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+      <c r="I22" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>28</v>
       </c>
@@ -1224,19 +1310,25 @@
         <v>3</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F23" s="31">
         <v>3</v>
       </c>
-      <c r="G23" s="33" t="s">
-        <v>81</v>
+      <c r="G23" s="1">
+        <v>2</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+        <v>96</v>
+      </c>
+      <c r="I23" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>29</v>
       </c>
@@ -1244,25 +1336,31 @@
         <v>39</v>
       </c>
       <c r="C24" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="1">
         <v>3</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="F24" s="31">
-        <v>3</v>
-      </c>
-      <c r="G24" s="33" t="s">
-        <v>55</v>
+        <v>70</v>
+      </c>
+      <c r="F24" s="30">
+        <v>6</v>
+      </c>
+      <c r="G24" s="1">
+        <v>3</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+        <v>94</v>
+      </c>
+      <c r="I24" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>30</v>
       </c>
@@ -1276,19 +1374,25 @@
         <v>2</v>
       </c>
       <c r="E25" s="33" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F25" s="32">
         <v>2</v>
       </c>
-      <c r="G25" s="33" t="s">
-        <v>56</v>
+      <c r="G25" s="1">
+        <v>2</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+        <v>97</v>
+      </c>
+      <c r="I25" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>31</v>
       </c>
@@ -1302,19 +1406,25 @@
         <v>2</v>
       </c>
       <c r="E26" s="33" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F26" s="31">
         <v>4</v>
       </c>
-      <c r="G26" s="33" t="s">
-        <v>80</v>
+      <c r="G26" s="1">
+        <v>2</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+      <c r="I26" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>32</v>
       </c>
@@ -1328,19 +1438,25 @@
         <v>2</v>
       </c>
       <c r="E27" s="33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F27" s="32">
         <v>2</v>
       </c>
-      <c r="G27" s="33" t="s">
-        <v>79</v>
-      </c>
-      <c r="H27" s="33" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="G27" s="1">
+        <v>2</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I27" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="J27" s="33" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>42</v>
       </c>
@@ -1354,19 +1470,25 @@
         <v>3</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F28" s="30">
         <v>6</v>
       </c>
-      <c r="G28" s="33" t="s">
-        <v>78</v>
+      <c r="G28" s="1">
+        <v>2</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+      <c r="I28" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>43</v>
       </c>
@@ -1380,25 +1502,31 @@
         <v>2</v>
       </c>
       <c r="E29" s="33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F29" s="32">
         <v>2</v>
       </c>
-      <c r="G29" s="33" t="s">
-        <v>77</v>
+      <c r="G29" s="1">
+        <v>2</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+      <c r="I29" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="33" t="s">
-        <v>63</v>
-      </c>
       <c r="C30" s="1">
         <v>2</v>
       </c>
@@ -1406,16 +1534,22 @@
         <v>3</v>
       </c>
       <c r="E30" s="33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F30" s="30">
         <v>6</v>
       </c>
-      <c r="G30" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>59</v>
+      <c r="G30" s="1">
+        <v>2</v>
+      </c>
+      <c r="H30" s="33" t="s">
+        <v>102</v>
+      </c>
+      <c r="I30" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>